<commit_message>
Update SD2 project files and add new content
</commit_message>
<xml_diff>
--- a/docs/Extras/SD2_S26/Bill-of-Materials-and-Budget/PRP BOM.xlsx
+++ b/docs/Extras/SD2_S26/Bill-of-Materials-and-Budget/PRP BOM.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="B/iAIK3GpbSqCLQ+5L0IKfjR2gVWE6goiiLjNdcYrgE="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="QrfrTFkwJtSt/lF6YwUUOm/EXgXr7yu5Z7fZOHJT9PE="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="292">
   <si>
     <t>Semester 1 Purchasing</t>
   </si>
@@ -843,6 +843,21 @@
     <t>LIPOLY BATTERY CHARGER W/USB C</t>
   </si>
   <si>
+    <t>1568-15217-ND</t>
+  </si>
+  <si>
+    <t>MCP73833 - Battery Charger Power Management Evaluation Board</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3.3 µH Shielded Multilayer Inductor 700 mA 438mOhm Max 0603 (1608 Metric)</t>
+  </si>
+  <si>
+    <t>2019-RK73B1JTTD203JCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 20 kOhms ±5% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
+  </si>
+  <si>
     <t>Total Spent</t>
   </si>
   <si>
@@ -862,6 +877,21 @@
   </si>
   <si>
     <t>Remaining Budget</t>
+  </si>
+  <si>
+    <t>Budget Breakdown</t>
+  </si>
+  <si>
+    <t>Electrical</t>
+  </si>
+  <si>
+    <t>Computer</t>
+  </si>
+  <si>
+    <t>Mechanical</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
@@ -871,7 +901,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -896,6 +926,11 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="8.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <sz val="12.0"/>
       <color theme="1"/>
       <name val="Aptos"/>
@@ -904,11 +939,6 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
     </font>
     <font>
       <strike/>
@@ -927,17 +957,22 @@
       <name val="Arial"/>
     </font>
     <font>
-      <b/>
       <sz val="8.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <color theme="1"/>
       <name val="Times New Roman"/>
     </font>
+    <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -952,14 +987,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
-        <bgColor rgb="FF00FF00"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1119,7 +1148,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="49">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1140,10 +1169,10 @@
     <xf borderId="4" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="4" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1160,35 +1189,45 @@
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="6" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="4" fillId="5" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="4" fillId="3" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="3" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="4" fillId="5" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="4" fillId="3" fontId="3" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="4" fillId="3" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="3" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="3" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="8" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="4" fillId="3" fontId="8" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="3" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="11" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1213,6 +1252,16 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="12" fillId="0" fontId="12" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="1" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="4" fillId="0" fontId="10" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1279,12 +1328,12 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$C$125:$C$128</c:f>
+              <c:f>Sheet1!$C$129:$C$132</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$125:$D$128</c:f>
+              <c:f>Sheet1!$D$129:$D$132</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -1311,13 +1360,115 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+  <c:chart>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$D$138</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="00FF00"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$C$139:$C$142</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$D$139:$D$142</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>123</xdr:row>
+      <xdr:row>127</xdr:row>
       <xdr:rowOff>28575</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3629025" cy="3533775"/>
@@ -1333,6 +1484,31 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1504950</xdr:colOff>
+      <xdr:row>135</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3448050" cy="2133600"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1543560228" name="Chart 2" title="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1616,7 +1792,7 @@
       <c r="F5" s="6">
         <v>6.48</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="7">
         <f t="shared" si="1"/>
         <v>19.44</v>
       </c>
@@ -1635,7 +1811,7 @@
       <c r="F6" s="6">
         <v>19.95</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="7">
         <f t="shared" si="1"/>
         <v>199.5</v>
       </c>
@@ -1656,7 +1832,7 @@
       <c r="F7" s="6">
         <v>4.18</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="7">
         <f t="shared" si="1"/>
         <v>29.26</v>
       </c>
@@ -1719,7 +1895,7 @@
       <c r="F10" s="6">
         <v>1.98</v>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="7">
         <f t="shared" si="1"/>
         <v>19.8</v>
       </c>
@@ -1759,7 +1935,7 @@
       <c r="F12" s="6">
         <v>1.24</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="7">
         <f t="shared" si="1"/>
         <v>12.4</v>
       </c>
@@ -1816,7 +1992,7 @@
       <c r="F15" s="6">
         <v>21.99</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="7">
         <f t="shared" si="1"/>
         <v>43.98</v>
       </c>
@@ -1835,7 +2011,7 @@
       <c r="F16" s="6">
         <v>7.99</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="7">
         <f t="shared" si="1"/>
         <v>7.99</v>
       </c>
@@ -1865,13 +2041,13 @@
       <c r="B18" s="5">
         <v>10.0</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="8" t="s">
         <v>41</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" s="9" t="s">
         <v>43</v>
       </c>
       <c r="F18" s="6">
@@ -1886,7 +2062,7 @@
       <c r="B19" s="5">
         <v>10.0</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D19" s="5" t="s">
@@ -2594,7 +2770,7 @@
       <c r="F54" s="6">
         <v>106.9</v>
       </c>
-      <c r="G54" s="6">
+      <c r="G54" s="7">
         <f t="shared" si="2"/>
         <v>106.9</v>
       </c>
@@ -2613,7 +2789,7 @@
       <c r="F55" s="6">
         <v>4.75</v>
       </c>
-      <c r="G55" s="6">
+      <c r="G55" s="7">
         <f t="shared" si="2"/>
         <v>47.5</v>
       </c>
@@ -2632,7 +2808,7 @@
       <c r="F56" s="6">
         <v>70.67</v>
       </c>
-      <c r="G56" s="8">
+      <c r="G56" s="7">
         <f t="shared" si="2"/>
         <v>70.67</v>
       </c>
@@ -2653,7 +2829,7 @@
       <c r="F57" s="6">
         <v>0.85</v>
       </c>
-      <c r="G57" s="6">
+      <c r="G57" s="7">
         <f t="shared" si="2"/>
         <v>8.5</v>
       </c>
@@ -2674,7 +2850,7 @@
       <c r="F58" s="6">
         <v>0.09</v>
       </c>
-      <c r="G58" s="6">
+      <c r="G58" s="7">
         <f t="shared" si="2"/>
         <v>1.8</v>
       </c>
@@ -2800,7 +2976,7 @@
       <c r="F64" s="6">
         <v>1.871</v>
       </c>
-      <c r="G64" s="6">
+      <c r="G64" s="7">
         <f t="shared" si="2"/>
         <v>18.71</v>
       </c>
@@ -3136,28 +3312,28 @@
         <v>0.18</v>
       </c>
       <c r="G82" s="20">
-        <f t="shared" ref="G82:G122" si="3">B82*F82</f>
+        <f t="shared" ref="G82:G126" si="3">B82*F82</f>
         <v>9.72</v>
       </c>
-      <c r="H82" s="17"/>
-      <c r="I82" s="17"/>
-      <c r="J82" s="17"/>
-      <c r="K82" s="17"/>
-      <c r="L82" s="17"/>
-      <c r="M82" s="17"/>
-      <c r="N82" s="17"/>
-      <c r="O82" s="17"/>
-      <c r="P82" s="17"/>
-      <c r="Q82" s="17"/>
-      <c r="R82" s="17"/>
-      <c r="S82" s="17"/>
-      <c r="T82" s="17"/>
-      <c r="U82" s="17"/>
-      <c r="V82" s="17"/>
-      <c r="W82" s="17"/>
-      <c r="X82" s="17"/>
-      <c r="Y82" s="17"/>
-      <c r="Z82" s="17"/>
+      <c r="H82" s="21"/>
+      <c r="I82" s="21"/>
+      <c r="J82" s="21"/>
+      <c r="K82" s="21"/>
+      <c r="L82" s="21"/>
+      <c r="M82" s="21"/>
+      <c r="N82" s="21"/>
+      <c r="O82" s="21"/>
+      <c r="P82" s="21"/>
+      <c r="Q82" s="21"/>
+      <c r="R82" s="21"/>
+      <c r="S82" s="21"/>
+      <c r="T82" s="21"/>
+      <c r="U82" s="21"/>
+      <c r="V82" s="21"/>
+      <c r="W82" s="21"/>
+      <c r="X82" s="21"/>
+      <c r="Y82" s="21"/>
+      <c r="Z82" s="21"/>
     </row>
     <row r="83" ht="14.25" customHeight="1">
       <c r="A83" s="17"/>
@@ -3173,32 +3349,32 @@
       <c r="E83" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="F83" s="21">
+      <c r="F83" s="22">
         <v>0.1</v>
       </c>
       <c r="G83" s="20">
         <f t="shared" si="3"/>
         <v>2.4</v>
       </c>
-      <c r="H83" s="17"/>
-      <c r="I83" s="17"/>
-      <c r="J83" s="17"/>
-      <c r="K83" s="17"/>
-      <c r="L83" s="17"/>
-      <c r="M83" s="17"/>
-      <c r="N83" s="17"/>
-      <c r="O83" s="17"/>
-      <c r="P83" s="17"/>
-      <c r="Q83" s="17"/>
-      <c r="R83" s="17"/>
-      <c r="S83" s="17"/>
-      <c r="T83" s="17"/>
-      <c r="U83" s="17"/>
-      <c r="V83" s="17"/>
-      <c r="W83" s="17"/>
-      <c r="X83" s="17"/>
-      <c r="Y83" s="17"/>
-      <c r="Z83" s="17"/>
+      <c r="H83" s="21"/>
+      <c r="I83" s="21"/>
+      <c r="J83" s="21"/>
+      <c r="K83" s="21"/>
+      <c r="L83" s="21"/>
+      <c r="M83" s="21"/>
+      <c r="N83" s="21"/>
+      <c r="O83" s="21"/>
+      <c r="P83" s="21"/>
+      <c r="Q83" s="21"/>
+      <c r="R83" s="21"/>
+      <c r="S83" s="21"/>
+      <c r="T83" s="21"/>
+      <c r="U83" s="21"/>
+      <c r="V83" s="21"/>
+      <c r="W83" s="21"/>
+      <c r="X83" s="21"/>
+      <c r="Y83" s="21"/>
+      <c r="Z83" s="21"/>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="17"/>
@@ -3211,7 +3387,7 @@
       <c r="D84" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="E84" s="22" t="s">
+      <c r="E84" s="23" t="s">
         <v>195</v>
       </c>
       <c r="F84" s="20">
@@ -3221,25 +3397,25 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="H84" s="17"/>
-      <c r="I84" s="17"/>
-      <c r="J84" s="17"/>
-      <c r="K84" s="17"/>
-      <c r="L84" s="17"/>
-      <c r="M84" s="17"/>
-      <c r="N84" s="17"/>
-      <c r="O84" s="17"/>
-      <c r="P84" s="17"/>
-      <c r="Q84" s="17"/>
-      <c r="R84" s="17"/>
-      <c r="S84" s="17"/>
-      <c r="T84" s="17"/>
-      <c r="U84" s="17"/>
-      <c r="V84" s="17"/>
-      <c r="W84" s="17"/>
-      <c r="X84" s="17"/>
-      <c r="Y84" s="17"/>
-      <c r="Z84" s="17"/>
+      <c r="H84" s="21"/>
+      <c r="I84" s="21"/>
+      <c r="J84" s="21"/>
+      <c r="K84" s="21"/>
+      <c r="L84" s="21"/>
+      <c r="M84" s="21"/>
+      <c r="N84" s="21"/>
+      <c r="O84" s="21"/>
+      <c r="P84" s="21"/>
+      <c r="Q84" s="21"/>
+      <c r="R84" s="21"/>
+      <c r="S84" s="21"/>
+      <c r="T84" s="21"/>
+      <c r="U84" s="21"/>
+      <c r="V84" s="21"/>
+      <c r="W84" s="21"/>
+      <c r="X84" s="21"/>
+      <c r="Y84" s="21"/>
+      <c r="Z84" s="21"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="17"/>
@@ -3252,7 +3428,7 @@
       <c r="D85" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="E85" s="22" t="s">
+      <c r="E85" s="23" t="s">
         <v>197</v>
       </c>
       <c r="F85" s="20">
@@ -3262,25 +3438,25 @@
         <f t="shared" si="3"/>
         <v>0.85</v>
       </c>
-      <c r="H85" s="17"/>
-      <c r="I85" s="17"/>
-      <c r="J85" s="17"/>
-      <c r="K85" s="17"/>
-      <c r="L85" s="17"/>
-      <c r="M85" s="17"/>
-      <c r="N85" s="17"/>
-      <c r="O85" s="17"/>
-      <c r="P85" s="17"/>
-      <c r="Q85" s="17"/>
-      <c r="R85" s="17"/>
-      <c r="S85" s="17"/>
-      <c r="T85" s="17"/>
-      <c r="U85" s="17"/>
-      <c r="V85" s="17"/>
-      <c r="W85" s="17"/>
-      <c r="X85" s="17"/>
-      <c r="Y85" s="17"/>
-      <c r="Z85" s="17"/>
+      <c r="H85" s="21"/>
+      <c r="I85" s="21"/>
+      <c r="J85" s="21"/>
+      <c r="K85" s="21"/>
+      <c r="L85" s="21"/>
+      <c r="M85" s="21"/>
+      <c r="N85" s="21"/>
+      <c r="O85" s="21"/>
+      <c r="P85" s="21"/>
+      <c r="Q85" s="21"/>
+      <c r="R85" s="21"/>
+      <c r="S85" s="21"/>
+      <c r="T85" s="21"/>
+      <c r="U85" s="21"/>
+      <c r="V85" s="21"/>
+      <c r="W85" s="21"/>
+      <c r="X85" s="21"/>
+      <c r="Y85" s="21"/>
+      <c r="Z85" s="21"/>
     </row>
     <row r="86" ht="14.25" customHeight="1">
       <c r="A86" s="17"/>
@@ -3290,7 +3466,7 @@
       <c r="C86" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="D86" s="22" t="s">
+      <c r="D86" s="23" t="s">
         <v>198</v>
       </c>
       <c r="E86" s="18" t="s">
@@ -3303,25 +3479,25 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="H86" s="17"/>
-      <c r="I86" s="17"/>
-      <c r="J86" s="17"/>
-      <c r="K86" s="17"/>
-      <c r="L86" s="17"/>
-      <c r="M86" s="17"/>
-      <c r="N86" s="17"/>
-      <c r="O86" s="17"/>
-      <c r="P86" s="17"/>
-      <c r="Q86" s="17"/>
-      <c r="R86" s="17"/>
-      <c r="S86" s="17"/>
-      <c r="T86" s="17"/>
-      <c r="U86" s="17"/>
-      <c r="V86" s="17"/>
-      <c r="W86" s="17"/>
-      <c r="X86" s="17"/>
-      <c r="Y86" s="17"/>
-      <c r="Z86" s="17"/>
+      <c r="H86" s="21"/>
+      <c r="I86" s="21"/>
+      <c r="J86" s="21"/>
+      <c r="K86" s="21"/>
+      <c r="L86" s="21"/>
+      <c r="M86" s="21"/>
+      <c r="N86" s="21"/>
+      <c r="O86" s="21"/>
+      <c r="P86" s="21"/>
+      <c r="Q86" s="21"/>
+      <c r="R86" s="21"/>
+      <c r="S86" s="21"/>
+      <c r="T86" s="21"/>
+      <c r="U86" s="21"/>
+      <c r="V86" s="21"/>
+      <c r="W86" s="21"/>
+      <c r="X86" s="21"/>
+      <c r="Y86" s="21"/>
+      <c r="Z86" s="21"/>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="17"/>
@@ -3331,10 +3507,10 @@
       <c r="C87" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="D87" s="22" t="s">
+      <c r="D87" s="23" t="s">
         <v>200</v>
       </c>
-      <c r="E87" s="22" t="s">
+      <c r="E87" s="23" t="s">
         <v>201</v>
       </c>
       <c r="F87" s="20">
@@ -3344,25 +3520,25 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="H87" s="17"/>
-      <c r="I87" s="17"/>
-      <c r="J87" s="17"/>
-      <c r="K87" s="17"/>
-      <c r="L87" s="17"/>
-      <c r="M87" s="17"/>
-      <c r="N87" s="17"/>
-      <c r="O87" s="17"/>
-      <c r="P87" s="17"/>
-      <c r="Q87" s="17"/>
-      <c r="R87" s="17"/>
-      <c r="S87" s="17"/>
-      <c r="T87" s="17"/>
-      <c r="U87" s="17"/>
-      <c r="V87" s="17"/>
-      <c r="W87" s="17"/>
-      <c r="X87" s="17"/>
-      <c r="Y87" s="17"/>
-      <c r="Z87" s="17"/>
+      <c r="H87" s="21"/>
+      <c r="I87" s="21"/>
+      <c r="J87" s="21"/>
+      <c r="K87" s="21"/>
+      <c r="L87" s="21"/>
+      <c r="M87" s="21"/>
+      <c r="N87" s="21"/>
+      <c r="O87" s="21"/>
+      <c r="P87" s="21"/>
+      <c r="Q87" s="21"/>
+      <c r="R87" s="21"/>
+      <c r="S87" s="21"/>
+      <c r="T87" s="21"/>
+      <c r="U87" s="21"/>
+      <c r="V87" s="21"/>
+      <c r="W87" s="21"/>
+      <c r="X87" s="21"/>
+      <c r="Y87" s="21"/>
+      <c r="Z87" s="21"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="17"/>
@@ -3385,25 +3561,25 @@
         <f t="shared" si="3"/>
         <v>4.45</v>
       </c>
-      <c r="H88" s="17"/>
-      <c r="I88" s="17"/>
-      <c r="J88" s="17"/>
-      <c r="K88" s="17"/>
-      <c r="L88" s="17"/>
-      <c r="M88" s="17"/>
-      <c r="N88" s="17"/>
-      <c r="O88" s="17"/>
-      <c r="P88" s="17"/>
-      <c r="Q88" s="17"/>
-      <c r="R88" s="17"/>
-      <c r="S88" s="17"/>
-      <c r="T88" s="17"/>
-      <c r="U88" s="17"/>
-      <c r="V88" s="17"/>
-      <c r="W88" s="17"/>
-      <c r="X88" s="17"/>
-      <c r="Y88" s="17"/>
-      <c r="Z88" s="17"/>
+      <c r="H88" s="21"/>
+      <c r="I88" s="21"/>
+      <c r="J88" s="21"/>
+      <c r="K88" s="21"/>
+      <c r="L88" s="21"/>
+      <c r="M88" s="21"/>
+      <c r="N88" s="21"/>
+      <c r="O88" s="21"/>
+      <c r="P88" s="21"/>
+      <c r="Q88" s="21"/>
+      <c r="R88" s="21"/>
+      <c r="S88" s="21"/>
+      <c r="T88" s="21"/>
+      <c r="U88" s="21"/>
+      <c r="V88" s="21"/>
+      <c r="W88" s="21"/>
+      <c r="X88" s="21"/>
+      <c r="Y88" s="21"/>
+      <c r="Z88" s="21"/>
     </row>
     <row r="89" ht="14.25" customHeight="1">
       <c r="A89" s="17"/>
@@ -3416,7 +3592,7 @@
       <c r="D89" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="E89" s="22" t="s">
+      <c r="E89" s="23" t="s">
         <v>204</v>
       </c>
       <c r="F89" s="20">
@@ -3426,25 +3602,25 @@
         <f t="shared" si="3"/>
         <v>3.4</v>
       </c>
-      <c r="H89" s="17"/>
-      <c r="I89" s="17"/>
-      <c r="J89" s="17"/>
-      <c r="K89" s="17"/>
-      <c r="L89" s="17"/>
-      <c r="M89" s="17"/>
-      <c r="N89" s="17"/>
-      <c r="O89" s="17"/>
-      <c r="P89" s="17"/>
-      <c r="Q89" s="17"/>
-      <c r="R89" s="17"/>
-      <c r="S89" s="17"/>
-      <c r="T89" s="17"/>
-      <c r="U89" s="17"/>
-      <c r="V89" s="17"/>
-      <c r="W89" s="17"/>
-      <c r="X89" s="17"/>
-      <c r="Y89" s="17"/>
-      <c r="Z89" s="17"/>
+      <c r="H89" s="21"/>
+      <c r="I89" s="21"/>
+      <c r="J89" s="21"/>
+      <c r="K89" s="21"/>
+      <c r="L89" s="21"/>
+      <c r="M89" s="21"/>
+      <c r="N89" s="21"/>
+      <c r="O89" s="21"/>
+      <c r="P89" s="21"/>
+      <c r="Q89" s="21"/>
+      <c r="R89" s="21"/>
+      <c r="S89" s="21"/>
+      <c r="T89" s="21"/>
+      <c r="U89" s="21"/>
+      <c r="V89" s="21"/>
+      <c r="W89" s="21"/>
+      <c r="X89" s="21"/>
+      <c r="Y89" s="21"/>
+      <c r="Z89" s="21"/>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="17"/>
@@ -3457,7 +3633,7 @@
       <c r="D90" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="E90" s="22" t="s">
+      <c r="E90" s="23" t="s">
         <v>206</v>
       </c>
       <c r="F90" s="20">
@@ -3467,47 +3643,48 @@
         <f t="shared" si="3"/>
         <v>7.2</v>
       </c>
-      <c r="H90" s="17"/>
-      <c r="I90" s="17"/>
-      <c r="J90" s="17"/>
-      <c r="K90" s="17"/>
-      <c r="L90" s="17"/>
-      <c r="M90" s="17"/>
-      <c r="N90" s="17"/>
-      <c r="O90" s="17"/>
-      <c r="P90" s="17"/>
-      <c r="Q90" s="17"/>
-      <c r="R90" s="17"/>
-      <c r="S90" s="17"/>
-      <c r="T90" s="17"/>
-      <c r="U90" s="17"/>
-      <c r="V90" s="17"/>
-      <c r="W90" s="17"/>
-      <c r="X90" s="17"/>
-      <c r="Y90" s="17"/>
-      <c r="Z90" s="17"/>
+      <c r="H90" s="21"/>
+      <c r="I90" s="21"/>
+      <c r="J90" s="21"/>
+      <c r="K90" s="21"/>
+      <c r="L90" s="21"/>
+      <c r="M90" s="21"/>
+      <c r="N90" s="21"/>
+      <c r="O90" s="21"/>
+      <c r="P90" s="21"/>
+      <c r="Q90" s="21"/>
+      <c r="R90" s="21"/>
+      <c r="S90" s="21"/>
+      <c r="T90" s="21"/>
+      <c r="U90" s="21"/>
+      <c r="V90" s="21"/>
+      <c r="W90" s="21"/>
+      <c r="X90" s="21"/>
+      <c r="Y90" s="21"/>
+      <c r="Z90" s="21"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
-      <c r="B91" s="23">
+      <c r="A91" s="17"/>
+      <c r="B91" s="24">
         <v>10.0</v>
       </c>
-      <c r="C91" s="24" t="s">
+      <c r="C91" s="25" t="s">
         <v>207</v>
       </c>
-      <c r="D91" s="24" t="s">
+      <c r="D91" s="25" t="s">
         <v>208</v>
       </c>
-      <c r="E91" s="23" t="s">
+      <c r="E91" s="24" t="s">
         <v>209</v>
       </c>
-      <c r="F91" s="25">
+      <c r="F91" s="26">
         <v>0.96</v>
       </c>
-      <c r="G91" s="25">
+      <c r="G91" s="26">
         <f t="shared" si="3"/>
         <v>9.6</v>
       </c>
-      <c r="H91" s="26" t="s">
+      <c r="H91" s="27" t="s">
         <v>210</v>
       </c>
     </row>
@@ -3532,25 +3709,25 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="H92" s="17"/>
-      <c r="I92" s="17"/>
-      <c r="J92" s="17"/>
-      <c r="K92" s="17"/>
-      <c r="L92" s="17"/>
-      <c r="M92" s="17"/>
-      <c r="N92" s="17"/>
-      <c r="O92" s="17"/>
-      <c r="P92" s="17"/>
-      <c r="Q92" s="17"/>
-      <c r="R92" s="17"/>
-      <c r="S92" s="17"/>
-      <c r="T92" s="17"/>
-      <c r="U92" s="17"/>
-      <c r="V92" s="17"/>
-      <c r="W92" s="17"/>
-      <c r="X92" s="17"/>
-      <c r="Y92" s="17"/>
-      <c r="Z92" s="17"/>
+      <c r="H92" s="21"/>
+      <c r="I92" s="21"/>
+      <c r="J92" s="21"/>
+      <c r="K92" s="21"/>
+      <c r="L92" s="21"/>
+      <c r="M92" s="21"/>
+      <c r="N92" s="21"/>
+      <c r="O92" s="21"/>
+      <c r="P92" s="21"/>
+      <c r="Q92" s="21"/>
+      <c r="R92" s="21"/>
+      <c r="S92" s="21"/>
+      <c r="T92" s="21"/>
+      <c r="U92" s="21"/>
+      <c r="V92" s="21"/>
+      <c r="W92" s="21"/>
+      <c r="X92" s="21"/>
+      <c r="Y92" s="21"/>
+      <c r="Z92" s="21"/>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="17"/>
@@ -3573,25 +3750,25 @@
         <f t="shared" si="3"/>
         <v>1.2</v>
       </c>
-      <c r="H93" s="17"/>
-      <c r="I93" s="17"/>
-      <c r="J93" s="17"/>
-      <c r="K93" s="17"/>
-      <c r="L93" s="17"/>
-      <c r="M93" s="17"/>
-      <c r="N93" s="17"/>
-      <c r="O93" s="17"/>
-      <c r="P93" s="17"/>
-      <c r="Q93" s="17"/>
-      <c r="R93" s="17"/>
-      <c r="S93" s="17"/>
-      <c r="T93" s="17"/>
-      <c r="U93" s="17"/>
-      <c r="V93" s="17"/>
-      <c r="W93" s="17"/>
-      <c r="X93" s="17"/>
-      <c r="Y93" s="17"/>
-      <c r="Z93" s="17"/>
+      <c r="H93" s="21"/>
+      <c r="I93" s="21"/>
+      <c r="J93" s="21"/>
+      <c r="K93" s="21"/>
+      <c r="L93" s="21"/>
+      <c r="M93" s="21"/>
+      <c r="N93" s="21"/>
+      <c r="O93" s="21"/>
+      <c r="P93" s="21"/>
+      <c r="Q93" s="21"/>
+      <c r="R93" s="21"/>
+      <c r="S93" s="21"/>
+      <c r="T93" s="21"/>
+      <c r="U93" s="21"/>
+      <c r="V93" s="21"/>
+      <c r="W93" s="21"/>
+      <c r="X93" s="21"/>
+      <c r="Y93" s="21"/>
+      <c r="Z93" s="21"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="17"/>
@@ -3614,25 +3791,25 @@
         <f t="shared" si="3"/>
         <v>1.8</v>
       </c>
-      <c r="H94" s="17"/>
-      <c r="I94" s="17"/>
-      <c r="J94" s="17"/>
-      <c r="K94" s="17"/>
-      <c r="L94" s="17"/>
-      <c r="M94" s="17"/>
-      <c r="N94" s="17"/>
-      <c r="O94" s="17"/>
-      <c r="P94" s="17"/>
-      <c r="Q94" s="17"/>
-      <c r="R94" s="17"/>
-      <c r="S94" s="17"/>
-      <c r="T94" s="17"/>
-      <c r="U94" s="17"/>
-      <c r="V94" s="17"/>
-      <c r="W94" s="17"/>
-      <c r="X94" s="17"/>
-      <c r="Y94" s="17"/>
-      <c r="Z94" s="17"/>
+      <c r="H94" s="21"/>
+      <c r="I94" s="21"/>
+      <c r="J94" s="21"/>
+      <c r="K94" s="21"/>
+      <c r="L94" s="21"/>
+      <c r="M94" s="21"/>
+      <c r="N94" s="21"/>
+      <c r="O94" s="21"/>
+      <c r="P94" s="21"/>
+      <c r="Q94" s="21"/>
+      <c r="R94" s="21"/>
+      <c r="S94" s="21"/>
+      <c r="T94" s="21"/>
+      <c r="U94" s="21"/>
+      <c r="V94" s="21"/>
+      <c r="W94" s="21"/>
+      <c r="X94" s="21"/>
+      <c r="Y94" s="21"/>
+      <c r="Z94" s="21"/>
     </row>
     <row r="95" ht="14.25" customHeight="1">
       <c r="A95" s="17"/>
@@ -3655,25 +3832,25 @@
         <f t="shared" si="3"/>
         <v>0.55</v>
       </c>
-      <c r="H95" s="17"/>
-      <c r="I95" s="17"/>
-      <c r="J95" s="17"/>
-      <c r="K95" s="17"/>
-      <c r="L95" s="17"/>
-      <c r="M95" s="17"/>
-      <c r="N95" s="17"/>
-      <c r="O95" s="17"/>
-      <c r="P95" s="17"/>
-      <c r="Q95" s="17"/>
-      <c r="R95" s="17"/>
-      <c r="S95" s="17"/>
-      <c r="T95" s="17"/>
-      <c r="U95" s="17"/>
-      <c r="V95" s="17"/>
-      <c r="W95" s="17"/>
-      <c r="X95" s="17"/>
-      <c r="Y95" s="17"/>
-      <c r="Z95" s="17"/>
+      <c r="H95" s="21"/>
+      <c r="I95" s="21"/>
+      <c r="J95" s="21"/>
+      <c r="K95" s="21"/>
+      <c r="L95" s="21"/>
+      <c r="M95" s="21"/>
+      <c r="N95" s="21"/>
+      <c r="O95" s="21"/>
+      <c r="P95" s="21"/>
+      <c r="Q95" s="21"/>
+      <c r="R95" s="21"/>
+      <c r="S95" s="21"/>
+      <c r="T95" s="21"/>
+      <c r="U95" s="21"/>
+      <c r="V95" s="21"/>
+      <c r="W95" s="21"/>
+      <c r="X95" s="21"/>
+      <c r="Y95" s="21"/>
+      <c r="Z95" s="21"/>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="17"/>
@@ -3696,25 +3873,25 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="H96" s="17"/>
-      <c r="I96" s="17"/>
-      <c r="J96" s="17"/>
-      <c r="K96" s="17"/>
-      <c r="L96" s="17"/>
-      <c r="M96" s="17"/>
-      <c r="N96" s="17"/>
-      <c r="O96" s="17"/>
-      <c r="P96" s="17"/>
-      <c r="Q96" s="17"/>
-      <c r="R96" s="17"/>
-      <c r="S96" s="17"/>
-      <c r="T96" s="17"/>
-      <c r="U96" s="17"/>
-      <c r="V96" s="17"/>
-      <c r="W96" s="17"/>
-      <c r="X96" s="17"/>
-      <c r="Y96" s="17"/>
-      <c r="Z96" s="17"/>
+      <c r="H96" s="21"/>
+      <c r="I96" s="21"/>
+      <c r="J96" s="21"/>
+      <c r="K96" s="21"/>
+      <c r="L96" s="21"/>
+      <c r="M96" s="21"/>
+      <c r="N96" s="21"/>
+      <c r="O96" s="21"/>
+      <c r="P96" s="21"/>
+      <c r="Q96" s="21"/>
+      <c r="R96" s="21"/>
+      <c r="S96" s="21"/>
+      <c r="T96" s="21"/>
+      <c r="U96" s="21"/>
+      <c r="V96" s="21"/>
+      <c r="W96" s="21"/>
+      <c r="X96" s="21"/>
+      <c r="Y96" s="21"/>
+      <c r="Z96" s="21"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="17"/>
@@ -3737,25 +3914,25 @@
         <f t="shared" si="3"/>
         <v>22.15</v>
       </c>
-      <c r="H97" s="17"/>
-      <c r="I97" s="17"/>
-      <c r="J97" s="17"/>
-      <c r="K97" s="17"/>
-      <c r="L97" s="17"/>
-      <c r="M97" s="17"/>
-      <c r="N97" s="17"/>
-      <c r="O97" s="17"/>
-      <c r="P97" s="17"/>
-      <c r="Q97" s="17"/>
-      <c r="R97" s="17"/>
-      <c r="S97" s="17"/>
-      <c r="T97" s="17"/>
-      <c r="U97" s="17"/>
-      <c r="V97" s="17"/>
-      <c r="W97" s="17"/>
-      <c r="X97" s="17"/>
-      <c r="Y97" s="17"/>
-      <c r="Z97" s="17"/>
+      <c r="H97" s="21"/>
+      <c r="I97" s="21"/>
+      <c r="J97" s="21"/>
+      <c r="K97" s="21"/>
+      <c r="L97" s="21"/>
+      <c r="M97" s="21"/>
+      <c r="N97" s="21"/>
+      <c r="O97" s="21"/>
+      <c r="P97" s="21"/>
+      <c r="Q97" s="21"/>
+      <c r="R97" s="21"/>
+      <c r="S97" s="21"/>
+      <c r="T97" s="21"/>
+      <c r="U97" s="21"/>
+      <c r="V97" s="21"/>
+      <c r="W97" s="21"/>
+      <c r="X97" s="21"/>
+      <c r="Y97" s="21"/>
+      <c r="Z97" s="21"/>
     </row>
     <row r="98" ht="14.25" customHeight="1">
       <c r="A98" s="17"/>
@@ -3778,25 +3955,25 @@
         <f t="shared" si="3"/>
         <v>10.95</v>
       </c>
-      <c r="H98" s="17"/>
-      <c r="I98" s="17"/>
-      <c r="J98" s="17"/>
-      <c r="K98" s="17"/>
-      <c r="L98" s="17"/>
-      <c r="M98" s="17"/>
-      <c r="N98" s="17"/>
-      <c r="O98" s="17"/>
-      <c r="P98" s="17"/>
-      <c r="Q98" s="17"/>
-      <c r="R98" s="17"/>
-      <c r="S98" s="17"/>
-      <c r="T98" s="17"/>
-      <c r="U98" s="17"/>
-      <c r="V98" s="17"/>
-      <c r="W98" s="17"/>
-      <c r="X98" s="17"/>
-      <c r="Y98" s="17"/>
-      <c r="Z98" s="17"/>
+      <c r="H98" s="21"/>
+      <c r="I98" s="21"/>
+      <c r="J98" s="21"/>
+      <c r="K98" s="21"/>
+      <c r="L98" s="21"/>
+      <c r="M98" s="21"/>
+      <c r="N98" s="21"/>
+      <c r="O98" s="21"/>
+      <c r="P98" s="21"/>
+      <c r="Q98" s="21"/>
+      <c r="R98" s="21"/>
+      <c r="S98" s="21"/>
+      <c r="T98" s="21"/>
+      <c r="U98" s="21"/>
+      <c r="V98" s="21"/>
+      <c r="W98" s="21"/>
+      <c r="X98" s="21"/>
+      <c r="Y98" s="21"/>
+      <c r="Z98" s="21"/>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="17"/>
@@ -3819,25 +3996,25 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="H99" s="17"/>
-      <c r="I99" s="17"/>
-      <c r="J99" s="17"/>
-      <c r="K99" s="17"/>
-      <c r="L99" s="17"/>
-      <c r="M99" s="17"/>
-      <c r="N99" s="17"/>
-      <c r="O99" s="17"/>
-      <c r="P99" s="17"/>
-      <c r="Q99" s="17"/>
-      <c r="R99" s="17"/>
-      <c r="S99" s="17"/>
-      <c r="T99" s="17"/>
-      <c r="U99" s="17"/>
-      <c r="V99" s="17"/>
-      <c r="W99" s="17"/>
-      <c r="X99" s="17"/>
-      <c r="Y99" s="17"/>
-      <c r="Z99" s="17"/>
+      <c r="H99" s="21"/>
+      <c r="I99" s="21"/>
+      <c r="J99" s="21"/>
+      <c r="K99" s="21"/>
+      <c r="L99" s="21"/>
+      <c r="M99" s="21"/>
+      <c r="N99" s="21"/>
+      <c r="O99" s="21"/>
+      <c r="P99" s="21"/>
+      <c r="Q99" s="21"/>
+      <c r="R99" s="21"/>
+      <c r="S99" s="21"/>
+      <c r="T99" s="21"/>
+      <c r="U99" s="21"/>
+      <c r="V99" s="21"/>
+      <c r="W99" s="21"/>
+      <c r="X99" s="21"/>
+      <c r="Y99" s="21"/>
+      <c r="Z99" s="21"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="17"/>
@@ -3860,25 +4037,25 @@
         <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
-      <c r="H100" s="17"/>
-      <c r="I100" s="17"/>
-      <c r="J100" s="17"/>
-      <c r="K100" s="17"/>
-      <c r="L100" s="17"/>
-      <c r="M100" s="17"/>
-      <c r="N100" s="17"/>
-      <c r="O100" s="17"/>
-      <c r="P100" s="17"/>
-      <c r="Q100" s="17"/>
-      <c r="R100" s="17"/>
-      <c r="S100" s="17"/>
-      <c r="T100" s="17"/>
-      <c r="U100" s="17"/>
-      <c r="V100" s="17"/>
-      <c r="W100" s="17"/>
-      <c r="X100" s="17"/>
-      <c r="Y100" s="17"/>
-      <c r="Z100" s="17"/>
+      <c r="H100" s="21"/>
+      <c r="I100" s="21"/>
+      <c r="J100" s="21"/>
+      <c r="K100" s="21"/>
+      <c r="L100" s="21"/>
+      <c r="M100" s="21"/>
+      <c r="N100" s="21"/>
+      <c r="O100" s="21"/>
+      <c r="P100" s="21"/>
+      <c r="Q100" s="21"/>
+      <c r="R100" s="21"/>
+      <c r="S100" s="21"/>
+      <c r="T100" s="21"/>
+      <c r="U100" s="21"/>
+      <c r="V100" s="21"/>
+      <c r="W100" s="21"/>
+      <c r="X100" s="21"/>
+      <c r="Y100" s="21"/>
+      <c r="Z100" s="21"/>
     </row>
     <row r="101" ht="14.25" customHeight="1">
       <c r="A101" s="17"/>
@@ -3901,25 +4078,25 @@
         <f t="shared" si="3"/>
         <v>4.2</v>
       </c>
-      <c r="H101" s="17"/>
-      <c r="I101" s="17"/>
-      <c r="J101" s="17"/>
-      <c r="K101" s="17"/>
-      <c r="L101" s="17"/>
-      <c r="M101" s="17"/>
-      <c r="N101" s="17"/>
-      <c r="O101" s="17"/>
-      <c r="P101" s="17"/>
-      <c r="Q101" s="17"/>
-      <c r="R101" s="17"/>
-      <c r="S101" s="17"/>
-      <c r="T101" s="17"/>
-      <c r="U101" s="17"/>
-      <c r="V101" s="17"/>
-      <c r="W101" s="17"/>
-      <c r="X101" s="17"/>
-      <c r="Y101" s="17"/>
-      <c r="Z101" s="17"/>
+      <c r="H101" s="21"/>
+      <c r="I101" s="21"/>
+      <c r="J101" s="21"/>
+      <c r="K101" s="21"/>
+      <c r="L101" s="21"/>
+      <c r="M101" s="21"/>
+      <c r="N101" s="21"/>
+      <c r="O101" s="21"/>
+      <c r="P101" s="21"/>
+      <c r="Q101" s="21"/>
+      <c r="R101" s="21"/>
+      <c r="S101" s="21"/>
+      <c r="T101" s="21"/>
+      <c r="U101" s="21"/>
+      <c r="V101" s="21"/>
+      <c r="W101" s="21"/>
+      <c r="X101" s="21"/>
+      <c r="Y101" s="21"/>
+      <c r="Z101" s="21"/>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="17"/>
@@ -3942,25 +4119,25 @@
         <f t="shared" si="3"/>
         <v>10.2</v>
       </c>
-      <c r="H102" s="17"/>
-      <c r="I102" s="17"/>
-      <c r="J102" s="17"/>
-      <c r="K102" s="17"/>
-      <c r="L102" s="17"/>
-      <c r="M102" s="17"/>
-      <c r="N102" s="17"/>
-      <c r="O102" s="17"/>
-      <c r="P102" s="17"/>
-      <c r="Q102" s="17"/>
-      <c r="R102" s="17"/>
-      <c r="S102" s="17"/>
-      <c r="T102" s="17"/>
-      <c r="U102" s="17"/>
-      <c r="V102" s="17"/>
-      <c r="W102" s="17"/>
-      <c r="X102" s="17"/>
-      <c r="Y102" s="17"/>
-      <c r="Z102" s="17"/>
+      <c r="H102" s="21"/>
+      <c r="I102" s="21"/>
+      <c r="J102" s="21"/>
+      <c r="K102" s="21"/>
+      <c r="L102" s="21"/>
+      <c r="M102" s="21"/>
+      <c r="N102" s="21"/>
+      <c r="O102" s="21"/>
+      <c r="P102" s="21"/>
+      <c r="Q102" s="21"/>
+      <c r="R102" s="21"/>
+      <c r="S102" s="21"/>
+      <c r="T102" s="21"/>
+      <c r="U102" s="21"/>
+      <c r="V102" s="21"/>
+      <c r="W102" s="21"/>
+      <c r="X102" s="21"/>
+      <c r="Y102" s="21"/>
+      <c r="Z102" s="21"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="17"/>
@@ -3983,25 +4160,25 @@
         <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
-      <c r="H103" s="17"/>
-      <c r="I103" s="17"/>
-      <c r="J103" s="17"/>
-      <c r="K103" s="17"/>
-      <c r="L103" s="17"/>
-      <c r="M103" s="17"/>
-      <c r="N103" s="17"/>
-      <c r="O103" s="17"/>
-      <c r="P103" s="17"/>
-      <c r="Q103" s="17"/>
-      <c r="R103" s="17"/>
-      <c r="S103" s="17"/>
-      <c r="T103" s="17"/>
-      <c r="U103" s="17"/>
-      <c r="V103" s="17"/>
-      <c r="W103" s="17"/>
-      <c r="X103" s="17"/>
-      <c r="Y103" s="17"/>
-      <c r="Z103" s="17"/>
+      <c r="H103" s="21"/>
+      <c r="I103" s="21"/>
+      <c r="J103" s="21"/>
+      <c r="K103" s="21"/>
+      <c r="L103" s="21"/>
+      <c r="M103" s="21"/>
+      <c r="N103" s="21"/>
+      <c r="O103" s="21"/>
+      <c r="P103" s="21"/>
+      <c r="Q103" s="21"/>
+      <c r="R103" s="21"/>
+      <c r="S103" s="21"/>
+      <c r="T103" s="21"/>
+      <c r="U103" s="21"/>
+      <c r="V103" s="21"/>
+      <c r="W103" s="21"/>
+      <c r="X103" s="21"/>
+      <c r="Y103" s="21"/>
+      <c r="Z103" s="21"/>
     </row>
     <row r="104" ht="14.25" customHeight="1">
       <c r="A104" s="17"/>
@@ -4024,25 +4201,25 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="H104" s="17"/>
-      <c r="I104" s="17"/>
-      <c r="J104" s="17"/>
-      <c r="K104" s="17"/>
-      <c r="L104" s="17"/>
-      <c r="M104" s="17"/>
-      <c r="N104" s="17"/>
-      <c r="O104" s="17"/>
-      <c r="P104" s="17"/>
-      <c r="Q104" s="17"/>
-      <c r="R104" s="17"/>
-      <c r="S104" s="17"/>
-      <c r="T104" s="17"/>
-      <c r="U104" s="17"/>
-      <c r="V104" s="17"/>
-      <c r="W104" s="17"/>
-      <c r="X104" s="17"/>
-      <c r="Y104" s="17"/>
-      <c r="Z104" s="17"/>
+      <c r="H104" s="21"/>
+      <c r="I104" s="21"/>
+      <c r="J104" s="21"/>
+      <c r="K104" s="21"/>
+      <c r="L104" s="21"/>
+      <c r="M104" s="21"/>
+      <c r="N104" s="21"/>
+      <c r="O104" s="21"/>
+      <c r="P104" s="21"/>
+      <c r="Q104" s="21"/>
+      <c r="R104" s="21"/>
+      <c r="S104" s="21"/>
+      <c r="T104" s="21"/>
+      <c r="U104" s="21"/>
+      <c r="V104" s="21"/>
+      <c r="W104" s="21"/>
+      <c r="X104" s="21"/>
+      <c r="Y104" s="21"/>
+      <c r="Z104" s="21"/>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="17"/>
@@ -4065,25 +4242,25 @@
         <f t="shared" si="3"/>
         <v>7.8</v>
       </c>
-      <c r="H105" s="17"/>
-      <c r="I105" s="17"/>
-      <c r="J105" s="17"/>
-      <c r="K105" s="17"/>
-      <c r="L105" s="17"/>
-      <c r="M105" s="17"/>
-      <c r="N105" s="17"/>
-      <c r="O105" s="17"/>
-      <c r="P105" s="17"/>
-      <c r="Q105" s="17"/>
-      <c r="R105" s="17"/>
-      <c r="S105" s="17"/>
-      <c r="T105" s="17"/>
-      <c r="U105" s="17"/>
-      <c r="V105" s="17"/>
-      <c r="W105" s="17"/>
-      <c r="X105" s="17"/>
-      <c r="Y105" s="17"/>
-      <c r="Z105" s="17"/>
+      <c r="H105" s="21"/>
+      <c r="I105" s="21"/>
+      <c r="J105" s="21"/>
+      <c r="K105" s="21"/>
+      <c r="L105" s="21"/>
+      <c r="M105" s="21"/>
+      <c r="N105" s="21"/>
+      <c r="O105" s="21"/>
+      <c r="P105" s="21"/>
+      <c r="Q105" s="21"/>
+      <c r="R105" s="21"/>
+      <c r="S105" s="21"/>
+      <c r="T105" s="21"/>
+      <c r="U105" s="21"/>
+      <c r="V105" s="21"/>
+      <c r="W105" s="21"/>
+      <c r="X105" s="21"/>
+      <c r="Y105" s="21"/>
+      <c r="Z105" s="21"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="17"/>
@@ -4106,25 +4283,25 @@
         <f t="shared" si="3"/>
         <v>14.75</v>
       </c>
-      <c r="H106" s="17"/>
-      <c r="I106" s="17"/>
-      <c r="J106" s="17"/>
-      <c r="K106" s="17"/>
-      <c r="L106" s="17"/>
-      <c r="M106" s="17"/>
-      <c r="N106" s="17"/>
-      <c r="O106" s="17"/>
-      <c r="P106" s="17"/>
-      <c r="Q106" s="17"/>
-      <c r="R106" s="17"/>
-      <c r="S106" s="17"/>
-      <c r="T106" s="17"/>
-      <c r="U106" s="17"/>
-      <c r="V106" s="17"/>
-      <c r="W106" s="17"/>
-      <c r="X106" s="17"/>
-      <c r="Y106" s="17"/>
-      <c r="Z106" s="17"/>
+      <c r="H106" s="21"/>
+      <c r="I106" s="21"/>
+      <c r="J106" s="21"/>
+      <c r="K106" s="21"/>
+      <c r="L106" s="21"/>
+      <c r="M106" s="21"/>
+      <c r="N106" s="21"/>
+      <c r="O106" s="21"/>
+      <c r="P106" s="21"/>
+      <c r="Q106" s="21"/>
+      <c r="R106" s="21"/>
+      <c r="S106" s="21"/>
+      <c r="T106" s="21"/>
+      <c r="U106" s="21"/>
+      <c r="V106" s="21"/>
+      <c r="W106" s="21"/>
+      <c r="X106" s="21"/>
+      <c r="Y106" s="21"/>
+      <c r="Z106" s="21"/>
     </row>
     <row r="107" ht="14.25" customHeight="1">
       <c r="A107" s="17"/>
@@ -4147,25 +4324,25 @@
         <f t="shared" si="3"/>
         <v>4.7</v>
       </c>
-      <c r="H107" s="17"/>
-      <c r="I107" s="17"/>
-      <c r="J107" s="17"/>
-      <c r="K107" s="17"/>
-      <c r="L107" s="17"/>
-      <c r="M107" s="17"/>
-      <c r="N107" s="17"/>
-      <c r="O107" s="17"/>
-      <c r="P107" s="17"/>
-      <c r="Q107" s="17"/>
-      <c r="R107" s="17"/>
-      <c r="S107" s="17"/>
-      <c r="T107" s="17"/>
-      <c r="U107" s="17"/>
-      <c r="V107" s="17"/>
-      <c r="W107" s="17"/>
-      <c r="X107" s="17"/>
-      <c r="Y107" s="17"/>
-      <c r="Z107" s="17"/>
+      <c r="H107" s="21"/>
+      <c r="I107" s="21"/>
+      <c r="J107" s="21"/>
+      <c r="K107" s="21"/>
+      <c r="L107" s="21"/>
+      <c r="M107" s="21"/>
+      <c r="N107" s="21"/>
+      <c r="O107" s="21"/>
+      <c r="P107" s="21"/>
+      <c r="Q107" s="21"/>
+      <c r="R107" s="21"/>
+      <c r="S107" s="21"/>
+      <c r="T107" s="21"/>
+      <c r="U107" s="21"/>
+      <c r="V107" s="21"/>
+      <c r="W107" s="21"/>
+      <c r="X107" s="21"/>
+      <c r="Y107" s="21"/>
+      <c r="Z107" s="21"/>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="17"/>
@@ -4188,25 +4365,25 @@
         <f t="shared" si="3"/>
         <v>23.7</v>
       </c>
-      <c r="H108" s="17"/>
-      <c r="I108" s="17"/>
-      <c r="J108" s="17"/>
-      <c r="K108" s="17"/>
-      <c r="L108" s="17"/>
-      <c r="M108" s="17"/>
-      <c r="N108" s="17"/>
-      <c r="O108" s="17"/>
-      <c r="P108" s="17"/>
-      <c r="Q108" s="17"/>
-      <c r="R108" s="17"/>
-      <c r="S108" s="17"/>
-      <c r="T108" s="17"/>
-      <c r="U108" s="17"/>
-      <c r="V108" s="17"/>
-      <c r="W108" s="17"/>
-      <c r="X108" s="17"/>
-      <c r="Y108" s="17"/>
-      <c r="Z108" s="17"/>
+      <c r="H108" s="21"/>
+      <c r="I108" s="21"/>
+      <c r="J108" s="21"/>
+      <c r="K108" s="21"/>
+      <c r="L108" s="21"/>
+      <c r="M108" s="21"/>
+      <c r="N108" s="21"/>
+      <c r="O108" s="21"/>
+      <c r="P108" s="21"/>
+      <c r="Q108" s="21"/>
+      <c r="R108" s="21"/>
+      <c r="S108" s="21"/>
+      <c r="T108" s="21"/>
+      <c r="U108" s="21"/>
+      <c r="V108" s="21"/>
+      <c r="W108" s="21"/>
+      <c r="X108" s="21"/>
+      <c r="Y108" s="21"/>
+      <c r="Z108" s="21"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="17"/>
@@ -4229,25 +4406,25 @@
         <f t="shared" si="3"/>
         <v>2.2</v>
       </c>
-      <c r="H109" s="17"/>
-      <c r="I109" s="17"/>
-      <c r="J109" s="17"/>
-      <c r="K109" s="17"/>
-      <c r="L109" s="17"/>
-      <c r="M109" s="17"/>
-      <c r="N109" s="17"/>
-      <c r="O109" s="17"/>
-      <c r="P109" s="17"/>
-      <c r="Q109" s="17"/>
-      <c r="R109" s="17"/>
-      <c r="S109" s="17"/>
-      <c r="T109" s="17"/>
-      <c r="U109" s="17"/>
-      <c r="V109" s="17"/>
-      <c r="W109" s="17"/>
-      <c r="X109" s="17"/>
-      <c r="Y109" s="17"/>
-      <c r="Z109" s="17"/>
+      <c r="H109" s="21"/>
+      <c r="I109" s="21"/>
+      <c r="J109" s="21"/>
+      <c r="K109" s="21"/>
+      <c r="L109" s="21"/>
+      <c r="M109" s="21"/>
+      <c r="N109" s="21"/>
+      <c r="O109" s="21"/>
+      <c r="P109" s="21"/>
+      <c r="Q109" s="21"/>
+      <c r="R109" s="21"/>
+      <c r="S109" s="21"/>
+      <c r="T109" s="21"/>
+      <c r="U109" s="21"/>
+      <c r="V109" s="21"/>
+      <c r="W109" s="21"/>
+      <c r="X109" s="21"/>
+      <c r="Y109" s="21"/>
+      <c r="Z109" s="21"/>
     </row>
     <row r="110" ht="14.25" customHeight="1">
       <c r="A110" s="17"/>
@@ -4270,25 +4447,25 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="H110" s="17"/>
-      <c r="I110" s="17"/>
-      <c r="J110" s="17"/>
-      <c r="K110" s="17"/>
-      <c r="L110" s="17"/>
-      <c r="M110" s="17"/>
-      <c r="N110" s="17"/>
-      <c r="O110" s="17"/>
-      <c r="P110" s="17"/>
-      <c r="Q110" s="17"/>
-      <c r="R110" s="17"/>
-      <c r="S110" s="17"/>
-      <c r="T110" s="17"/>
-      <c r="U110" s="17"/>
-      <c r="V110" s="17"/>
-      <c r="W110" s="17"/>
-      <c r="X110" s="17"/>
-      <c r="Y110" s="17"/>
-      <c r="Z110" s="17"/>
+      <c r="H110" s="21"/>
+      <c r="I110" s="21"/>
+      <c r="J110" s="21"/>
+      <c r="K110" s="21"/>
+      <c r="L110" s="21"/>
+      <c r="M110" s="21"/>
+      <c r="N110" s="21"/>
+      <c r="O110" s="21"/>
+      <c r="P110" s="21"/>
+      <c r="Q110" s="21"/>
+      <c r="R110" s="21"/>
+      <c r="S110" s="21"/>
+      <c r="T110" s="21"/>
+      <c r="U110" s="21"/>
+      <c r="V110" s="21"/>
+      <c r="W110" s="21"/>
+      <c r="X110" s="21"/>
+      <c r="Y110" s="21"/>
+      <c r="Z110" s="21"/>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="17"/>
@@ -4311,25 +4488,25 @@
         <f t="shared" si="3"/>
         <v>12.4</v>
       </c>
-      <c r="H111" s="17"/>
-      <c r="I111" s="17"/>
-      <c r="J111" s="17"/>
-      <c r="K111" s="17"/>
-      <c r="L111" s="17"/>
-      <c r="M111" s="17"/>
-      <c r="N111" s="17"/>
-      <c r="O111" s="17"/>
-      <c r="P111" s="17"/>
-      <c r="Q111" s="17"/>
-      <c r="R111" s="17"/>
-      <c r="S111" s="17"/>
-      <c r="T111" s="17"/>
-      <c r="U111" s="17"/>
-      <c r="V111" s="17"/>
-      <c r="W111" s="17"/>
-      <c r="X111" s="17"/>
-      <c r="Y111" s="17"/>
-      <c r="Z111" s="17"/>
+      <c r="H111" s="21"/>
+      <c r="I111" s="21"/>
+      <c r="J111" s="21"/>
+      <c r="K111" s="21"/>
+      <c r="L111" s="21"/>
+      <c r="M111" s="21"/>
+      <c r="N111" s="21"/>
+      <c r="O111" s="21"/>
+      <c r="P111" s="21"/>
+      <c r="Q111" s="21"/>
+      <c r="R111" s="21"/>
+      <c r="S111" s="21"/>
+      <c r="T111" s="21"/>
+      <c r="U111" s="21"/>
+      <c r="V111" s="21"/>
+      <c r="W111" s="21"/>
+      <c r="X111" s="21"/>
+      <c r="Y111" s="21"/>
+      <c r="Z111" s="21"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="17"/>
@@ -4352,25 +4529,25 @@
         <f t="shared" si="3"/>
         <v>2.2</v>
       </c>
-      <c r="H112" s="17"/>
-      <c r="I112" s="17"/>
-      <c r="J112" s="17"/>
-      <c r="K112" s="17"/>
-      <c r="L112" s="17"/>
-      <c r="M112" s="17"/>
-      <c r="N112" s="17"/>
-      <c r="O112" s="17"/>
-      <c r="P112" s="17"/>
-      <c r="Q112" s="17"/>
-      <c r="R112" s="17"/>
-      <c r="S112" s="17"/>
-      <c r="T112" s="17"/>
-      <c r="U112" s="17"/>
-      <c r="V112" s="17"/>
-      <c r="W112" s="17"/>
-      <c r="X112" s="17"/>
-      <c r="Y112" s="17"/>
-      <c r="Z112" s="17"/>
+      <c r="H112" s="21"/>
+      <c r="I112" s="21"/>
+      <c r="J112" s="21"/>
+      <c r="K112" s="21"/>
+      <c r="L112" s="21"/>
+      <c r="M112" s="21"/>
+      <c r="N112" s="21"/>
+      <c r="O112" s="21"/>
+      <c r="P112" s="21"/>
+      <c r="Q112" s="21"/>
+      <c r="R112" s="21"/>
+      <c r="S112" s="21"/>
+      <c r="T112" s="21"/>
+      <c r="U112" s="21"/>
+      <c r="V112" s="21"/>
+      <c r="W112" s="21"/>
+      <c r="X112" s="21"/>
+      <c r="Y112" s="21"/>
+      <c r="Z112" s="21"/>
     </row>
     <row r="113" ht="14.25" customHeight="1">
       <c r="A113" s="17"/>
@@ -4386,32 +4563,32 @@
       <c r="E113" s="18" t="s">
         <v>257</v>
       </c>
-      <c r="F113" s="21">
+      <c r="F113" s="22">
         <v>0.1</v>
       </c>
       <c r="G113" s="20">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="H113" s="17"/>
-      <c r="I113" s="17"/>
-      <c r="J113" s="17"/>
-      <c r="K113" s="17"/>
-      <c r="L113" s="17"/>
-      <c r="M113" s="17"/>
-      <c r="N113" s="17"/>
-      <c r="O113" s="17"/>
-      <c r="P113" s="17"/>
-      <c r="Q113" s="17"/>
-      <c r="R113" s="17"/>
-      <c r="S113" s="17"/>
-      <c r="T113" s="17"/>
-      <c r="U113" s="17"/>
-      <c r="V113" s="17"/>
-      <c r="W113" s="17"/>
-      <c r="X113" s="17"/>
-      <c r="Y113" s="17"/>
-      <c r="Z113" s="17"/>
+      <c r="H113" s="21"/>
+      <c r="I113" s="21"/>
+      <c r="J113" s="21"/>
+      <c r="K113" s="21"/>
+      <c r="L113" s="21"/>
+      <c r="M113" s="21"/>
+      <c r="N113" s="21"/>
+      <c r="O113" s="21"/>
+      <c r="P113" s="21"/>
+      <c r="Q113" s="21"/>
+      <c r="R113" s="21"/>
+      <c r="S113" s="21"/>
+      <c r="T113" s="21"/>
+      <c r="U113" s="21"/>
+      <c r="V113" s="21"/>
+      <c r="W113" s="21"/>
+      <c r="X113" s="21"/>
+      <c r="Y113" s="21"/>
+      <c r="Z113" s="21"/>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="17"/>
@@ -4434,25 +4611,25 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="H114" s="17"/>
-      <c r="I114" s="17"/>
-      <c r="J114" s="17"/>
-      <c r="K114" s="17"/>
-      <c r="L114" s="17"/>
-      <c r="M114" s="17"/>
-      <c r="N114" s="17"/>
-      <c r="O114" s="17"/>
-      <c r="P114" s="17"/>
-      <c r="Q114" s="17"/>
-      <c r="R114" s="17"/>
-      <c r="S114" s="17"/>
-      <c r="T114" s="17"/>
-      <c r="U114" s="17"/>
-      <c r="V114" s="17"/>
-      <c r="W114" s="17"/>
-      <c r="X114" s="17"/>
-      <c r="Y114" s="17"/>
-      <c r="Z114" s="17"/>
+      <c r="H114" s="21"/>
+      <c r="I114" s="21"/>
+      <c r="J114" s="21"/>
+      <c r="K114" s="21"/>
+      <c r="L114" s="21"/>
+      <c r="M114" s="21"/>
+      <c r="N114" s="21"/>
+      <c r="O114" s="21"/>
+      <c r="P114" s="21"/>
+      <c r="Q114" s="21"/>
+      <c r="R114" s="21"/>
+      <c r="S114" s="21"/>
+      <c r="T114" s="21"/>
+      <c r="U114" s="21"/>
+      <c r="V114" s="21"/>
+      <c r="W114" s="21"/>
+      <c r="X114" s="21"/>
+      <c r="Y114" s="21"/>
+      <c r="Z114" s="21"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="17"/>
@@ -4475,25 +4652,25 @@
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="H115" s="17"/>
-      <c r="I115" s="17"/>
-      <c r="J115" s="17"/>
-      <c r="K115" s="17"/>
-      <c r="L115" s="17"/>
-      <c r="M115" s="17"/>
-      <c r="N115" s="17"/>
-      <c r="O115" s="17"/>
-      <c r="P115" s="17"/>
-      <c r="Q115" s="17"/>
-      <c r="R115" s="17"/>
-      <c r="S115" s="17"/>
-      <c r="T115" s="17"/>
-      <c r="U115" s="17"/>
-      <c r="V115" s="17"/>
-      <c r="W115" s="17"/>
-      <c r="X115" s="17"/>
-      <c r="Y115" s="17"/>
-      <c r="Z115" s="17"/>
+      <c r="H115" s="21"/>
+      <c r="I115" s="21"/>
+      <c r="J115" s="21"/>
+      <c r="K115" s="21"/>
+      <c r="L115" s="21"/>
+      <c r="M115" s="21"/>
+      <c r="N115" s="21"/>
+      <c r="O115" s="21"/>
+      <c r="P115" s="21"/>
+      <c r="Q115" s="21"/>
+      <c r="R115" s="21"/>
+      <c r="S115" s="21"/>
+      <c r="T115" s="21"/>
+      <c r="U115" s="21"/>
+      <c r="V115" s="21"/>
+      <c r="W115" s="21"/>
+      <c r="X115" s="21"/>
+      <c r="Y115" s="21"/>
+      <c r="Z115" s="21"/>
     </row>
     <row r="116" ht="14.25" customHeight="1">
       <c r="A116" s="17"/>
@@ -4516,25 +4693,25 @@
         <f t="shared" si="3"/>
         <v>7.95</v>
       </c>
-      <c r="H116" s="17"/>
-      <c r="I116" s="17"/>
-      <c r="J116" s="17"/>
-      <c r="K116" s="17"/>
-      <c r="L116" s="17"/>
-      <c r="M116" s="17"/>
-      <c r="N116" s="17"/>
-      <c r="O116" s="17"/>
-      <c r="P116" s="17"/>
-      <c r="Q116" s="17"/>
-      <c r="R116" s="17"/>
-      <c r="S116" s="17"/>
-      <c r="T116" s="17"/>
-      <c r="U116" s="17"/>
-      <c r="V116" s="17"/>
-      <c r="W116" s="17"/>
-      <c r="X116" s="17"/>
-      <c r="Y116" s="17"/>
-      <c r="Z116" s="17"/>
+      <c r="H116" s="21"/>
+      <c r="I116" s="21"/>
+      <c r="J116" s="21"/>
+      <c r="K116" s="21"/>
+      <c r="L116" s="21"/>
+      <c r="M116" s="21"/>
+      <c r="N116" s="21"/>
+      <c r="O116" s="21"/>
+      <c r="P116" s="21"/>
+      <c r="Q116" s="21"/>
+      <c r="R116" s="21"/>
+      <c r="S116" s="21"/>
+      <c r="T116" s="21"/>
+      <c r="U116" s="21"/>
+      <c r="V116" s="21"/>
+      <c r="W116" s="21"/>
+      <c r="X116" s="21"/>
+      <c r="Y116" s="21"/>
+      <c r="Z116" s="21"/>
     </row>
     <row r="117" ht="14.25" customHeight="1">
       <c r="A117" s="17"/>
@@ -4557,25 +4734,25 @@
         <f t="shared" si="3"/>
         <v>9.15</v>
       </c>
-      <c r="H117" s="17"/>
-      <c r="I117" s="17"/>
-      <c r="J117" s="17"/>
-      <c r="K117" s="17"/>
-      <c r="L117" s="17"/>
-      <c r="M117" s="17"/>
-      <c r="N117" s="17"/>
-      <c r="O117" s="17"/>
-      <c r="P117" s="17"/>
-      <c r="Q117" s="17"/>
-      <c r="R117" s="17"/>
-      <c r="S117" s="17"/>
-      <c r="T117" s="17"/>
-      <c r="U117" s="17"/>
-      <c r="V117" s="17"/>
-      <c r="W117" s="17"/>
-      <c r="X117" s="17"/>
-      <c r="Y117" s="17"/>
-      <c r="Z117" s="17"/>
+      <c r="H117" s="21"/>
+      <c r="I117" s="21"/>
+      <c r="J117" s="21"/>
+      <c r="K117" s="21"/>
+      <c r="L117" s="21"/>
+      <c r="M117" s="21"/>
+      <c r="N117" s="21"/>
+      <c r="O117" s="21"/>
+      <c r="P117" s="21"/>
+      <c r="Q117" s="21"/>
+      <c r="R117" s="21"/>
+      <c r="S117" s="21"/>
+      <c r="T117" s="21"/>
+      <c r="U117" s="21"/>
+      <c r="V117" s="21"/>
+      <c r="W117" s="21"/>
+      <c r="X117" s="21"/>
+      <c r="Y117" s="21"/>
+      <c r="Z117" s="21"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="B118" s="12">
@@ -4588,10 +4765,10 @@
       <c r="E118" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="F118" s="27">
+      <c r="F118" s="28">
         <v>4.75</v>
       </c>
-      <c r="G118" s="27">
+      <c r="G118" s="28">
         <f t="shared" si="3"/>
         <v>23.75</v>
       </c>
@@ -4607,10 +4784,10 @@
       <c r="E119" s="12" t="s">
         <v>269</v>
       </c>
-      <c r="F119" s="27">
+      <c r="F119" s="28">
         <v>35.72</v>
       </c>
-      <c r="G119" s="27">
+      <c r="G119" s="28">
         <f t="shared" si="3"/>
         <v>357.2</v>
       </c>
@@ -4626,10 +4803,10 @@
       <c r="E120" s="12" t="s">
         <v>271</v>
       </c>
-      <c r="F120" s="27">
+      <c r="F120" s="28">
         <v>216.8</v>
       </c>
-      <c r="G120" s="27">
+      <c r="G120" s="28">
         <f t="shared" si="3"/>
         <v>216.8</v>
       </c>
@@ -4645,127 +4822,242 @@
       <c r="E121" s="12" t="s">
         <v>272</v>
       </c>
-      <c r="F121" s="27">
+      <c r="F121" s="28">
         <v>68.07</v>
       </c>
-      <c r="G121" s="27">
+      <c r="G121" s="28">
         <f t="shared" si="3"/>
         <v>68.07</v>
       </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
-      <c r="B122" s="28">
+      <c r="B122" s="29">
         <v>2.0</v>
       </c>
-      <c r="C122" s="28">
+      <c r="C122" s="30">
         <v>4410.0</v>
       </c>
-      <c r="D122" s="28" t="s">
+      <c r="D122" s="29" t="s">
         <v>273</v>
       </c>
-      <c r="E122" s="28" t="s">
+      <c r="E122" s="29" t="s">
         <v>274</v>
       </c>
-      <c r="F122" s="29">
+      <c r="F122" s="31">
         <v>5.95</v>
       </c>
-      <c r="G122" s="27">
+      <c r="G122" s="28">
         <f t="shared" si="3"/>
         <v>11.9</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
-      <c r="F123" s="30" t="s">
+      <c r="B123" s="29">
+        <v>2.0</v>
+      </c>
+      <c r="C123" s="30">
+        <v>4410.0</v>
+      </c>
+      <c r="D123" s="32" t="s">
+        <v>273</v>
+      </c>
+      <c r="E123" s="32" t="s">
+        <v>274</v>
+      </c>
+      <c r="F123" s="31">
+        <v>5.95</v>
+      </c>
+      <c r="G123" s="28">
+        <f t="shared" si="3"/>
+        <v>11.9</v>
+      </c>
+    </row>
+    <row r="124" ht="14.25" customHeight="1">
+      <c r="B124" s="29">
+        <v>2.0</v>
+      </c>
+      <c r="C124" s="33">
+        <v>15217.0</v>
+      </c>
+      <c r="D124" s="32" t="s">
+        <v>275</v>
+      </c>
+      <c r="E124" s="32" t="s">
+        <v>276</v>
+      </c>
+      <c r="F124" s="31"/>
+      <c r="G124" s="28">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" ht="14.25" customHeight="1">
+      <c r="B125" s="29">
+        <v>10.0</v>
+      </c>
+      <c r="C125" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="D125" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="E125" s="32" t="s">
+        <v>277</v>
+      </c>
+      <c r="F125" s="31"/>
+      <c r="G125" s="28">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" ht="14.25" customHeight="1">
+      <c r="B126" s="29">
+        <v>20.0</v>
+      </c>
+      <c r="C126" s="32" t="s">
+        <v>260</v>
+      </c>
+      <c r="D126" s="32" t="s">
+        <v>278</v>
+      </c>
+      <c r="E126" s="32" t="s">
+        <v>279</v>
+      </c>
+      <c r="F126" s="31"/>
+      <c r="G126" s="28">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" ht="14.25" customHeight="1">
+      <c r="F127" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="G123" s="27">
-        <f>SUM(G83:G122)</f>
-        <v>858.52</v>
-      </c>
-    </row>
-    <row r="124" ht="14.25" customHeight="1">
-      <c r="C124" s="31" t="s">
-        <v>275</v>
-      </c>
-      <c r="D124" s="32"/>
-    </row>
-    <row r="125" ht="14.25" customHeight="1">
-      <c r="C125" s="33" t="s">
-        <v>276</v>
-      </c>
-      <c r="D125" s="34">
+      <c r="G127" s="28">
+        <f>SUM(G83:G126)</f>
+        <v>870.42</v>
+      </c>
+    </row>
+    <row r="128" ht="14.25" customHeight="1">
+      <c r="C128" s="35" t="s">
+        <v>280</v>
+      </c>
+      <c r="D128" s="36"/>
+    </row>
+    <row r="129" ht="14.25" customHeight="1">
+      <c r="C129" s="37" t="s">
+        <v>281</v>
+      </c>
+      <c r="D129" s="38">
         <f>SUM(G92:G122,G82:G90,G64:G77,G58,G57,G51:G55,G17:G46,G12,G10,G7,G6,G5)</f>
         <v>1957.48</v>
       </c>
     </row>
-    <row r="126" ht="14.25" customHeight="1">
-      <c r="C126" s="35" t="s">
-        <v>277</v>
-      </c>
-      <c r="D126" s="36">
+    <row r="130" ht="14.25" customHeight="1">
+      <c r="C130" s="39" t="s">
+        <v>282</v>
+      </c>
+      <c r="D130" s="40">
         <f>SUM(G63,G62,G61,G60,G59,G14,G11,G9,G8,G4,G13)</f>
         <v>827.05</v>
       </c>
     </row>
-    <row r="127" ht="14.25" customHeight="1">
-      <c r="C127" s="35" t="s">
-        <v>278</v>
-      </c>
-      <c r="D127" s="36">
+    <row r="131" ht="14.25" customHeight="1">
+      <c r="C131" s="39" t="s">
+        <v>283</v>
+      </c>
+      <c r="D131" s="40">
         <f>SUM(G56,G16,G15)</f>
         <v>122.64</v>
       </c>
-      <c r="F127" s="37">
+      <c r="F131" s="41">
         <f>sum(G92:G117)+sum(G122)+sum(G82:G90)</f>
         <v>192.82</v>
       </c>
     </row>
-    <row r="128" ht="14.25" customHeight="1">
-      <c r="C128" s="35" t="s">
-        <v>279</v>
-      </c>
-      <c r="D128" s="36">
+    <row r="132" ht="14.25" customHeight="1">
+      <c r="C132" s="39" t="s">
+        <v>284</v>
+      </c>
+      <c r="D132" s="40">
         <v>120.36</v>
       </c>
     </row>
-    <row r="129" ht="14.25" customHeight="1">
-      <c r="C129" s="35" t="s">
-        <v>275</v>
-      </c>
-      <c r="D129" s="38">
-        <f>SUM(D125,D126,D127,D128)-100.63</f>
+    <row r="133" ht="14.25" customHeight="1">
+      <c r="C133" s="39" t="s">
+        <v>280</v>
+      </c>
+      <c r="D133" s="42">
+        <f>SUM(D129,D130,D131,D132)-100.63</f>
         <v>2926.9</v>
       </c>
     </row>
-    <row r="130" ht="14.25" customHeight="1">
-      <c r="C130" s="35" t="s">
-        <v>280</v>
-      </c>
-      <c r="D130" s="36">
+    <row r="134" ht="14.25" customHeight="1">
+      <c r="C134" s="39" t="s">
+        <v>285</v>
+      </c>
+      <c r="D134" s="40">
         <v>3250.0</v>
       </c>
     </row>
-    <row r="131" ht="14.25" customHeight="1">
-      <c r="C131" s="39" t="s">
-        <v>281</v>
-      </c>
-      <c r="D131" s="40">
-        <f>D130-D129</f>
+    <row r="135" ht="14.25" customHeight="1">
+      <c r="C135" s="43" t="s">
+        <v>286</v>
+      </c>
+      <c r="D135" s="44">
+        <f>D134-D133</f>
         <v>323.1</v>
       </c>
     </row>
-    <row r="132" ht="14.25" customHeight="1"/>
-    <row r="133" ht="14.25" customHeight="1"/>
-    <row r="134" ht="14.25" customHeight="1"/>
-    <row r="135" ht="14.25" customHeight="1"/>
     <row r="136" ht="14.25" customHeight="1"/>
     <row r="137" ht="14.25" customHeight="1"/>
-    <row r="138" ht="14.25" customHeight="1"/>
-    <row r="139" ht="14.25" customHeight="1"/>
-    <row r="140" ht="14.25" customHeight="1"/>
-    <row r="141" ht="14.25" customHeight="1"/>
-    <row r="142" ht="14.25" customHeight="1"/>
-    <row r="143" ht="14.25" customHeight="1"/>
+    <row r="138" ht="14.25" customHeight="1">
+      <c r="C138" s="45" t="s">
+        <v>287</v>
+      </c>
+      <c r="D138" s="3"/>
+    </row>
+    <row r="139" ht="14.25" customHeight="1">
+      <c r="C139" s="46" t="s">
+        <v>288</v>
+      </c>
+      <c r="D139" s="47">
+        <f>D143-D142-D141-D140</f>
+        <v>1894.01</v>
+      </c>
+    </row>
+    <row r="140" ht="14.25" customHeight="1">
+      <c r="C140" s="46" t="s">
+        <v>289</v>
+      </c>
+      <c r="D140" s="48">
+        <v>827.05</v>
+      </c>
+    </row>
+    <row r="141" ht="14.25" customHeight="1">
+      <c r="C141" s="46" t="s">
+        <v>290</v>
+      </c>
+      <c r="D141" s="48">
+        <v>122.64</v>
+      </c>
+    </row>
+    <row r="142" ht="14.25" customHeight="1">
+      <c r="C142" s="46" t="s">
+        <v>284</v>
+      </c>
+      <c r="D142" s="48">
+        <v>120.36</v>
+      </c>
+    </row>
+    <row r="143" ht="14.25" customHeight="1">
+      <c r="C143" s="46" t="s">
+        <v>291</v>
+      </c>
+      <c r="D143" s="48">
+        <v>2964.06</v>
+      </c>
+    </row>
     <row r="144" ht="14.25" customHeight="1"/>
     <row r="145" ht="14.25" customHeight="1"/>
     <row r="146" ht="14.25" customHeight="1"/>
@@ -5623,12 +5915,17 @@
     <row r="998" ht="14.25" customHeight="1"/>
     <row r="999" ht="14.25" customHeight="1"/>
     <row r="1000" ht="14.25" customHeight="1"/>
+    <row r="1001" ht="14.25" customHeight="1"/>
+    <row r="1002" ht="14.25" customHeight="1"/>
+    <row r="1003" ht="14.25" customHeight="1"/>
+    <row r="1004" ht="14.25" customHeight="1"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B49:G49"/>
     <mergeCell ref="B80:G80"/>
-    <mergeCell ref="C124:D124"/>
+    <mergeCell ref="C128:D128"/>
+    <mergeCell ref="C138:D138"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>